<commit_message>
commit changes and updated the timeline
</commit_message>
<xml_diff>
--- a/docs/EduFlow AI Details.xlsx
+++ b/docs/EduFlow AI Details.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Personal Projects\EduFlowAI\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E63A1A4F-9E1A-45C8-8F46-6CD0F1B59778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BB4F1AC-B61D-41EE-A3A3-2B41CE325563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{92BD4C14-6350-41A2-989D-BE19952A9F2F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{92BD4C14-6350-41A2-989D-BE19952A9F2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Features" sheetId="2" r:id="rId2"/>
     <sheet name="Open Questions" sheetId="4" r:id="rId3"/>
-    <sheet name="EduFlow TimeLine" sheetId="5" r:id="rId4"/>
+    <sheet name="Color Theme " sheetId="6" r:id="rId4"/>
+    <sheet name="EduFlow TimeLine" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="130">
   <si>
     <t>EduFlow AI</t>
   </si>
@@ -84,9 +85,6 @@
     <t xml:space="preserve">Features </t>
   </si>
   <si>
-    <t xml:space="preserve">Phase </t>
-  </si>
-  <si>
     <t xml:space="preserve">Status </t>
   </si>
   <si>
@@ -192,43 +190,235 @@
     <t>S.No</t>
   </si>
   <si>
-    <t xml:space="preserve">Task </t>
-  </si>
-  <si>
     <t>Start Date</t>
   </si>
   <si>
-    <t xml:space="preserve">End Date </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creating Functional Requirement For the Project </t>
-  </si>
-  <si>
     <t>Requirement Phase</t>
   </si>
   <si>
     <t xml:space="preserve">EduFlow AI TimeLine </t>
   </si>
   <si>
-    <t xml:space="preserve">Rough Sketching of the project workflow </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI / UX Design using Google Stitch and Figma </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Designing Phase </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finalize the design of the project </t>
-  </si>
-  <si>
-    <t>Front End Development</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Database Structure </t>
-  </si>
-  <si>
     <t>Database Design</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Hex</t>
+  </si>
+  <si>
+    <t>Primary</t>
+  </si>
+  <si>
+    <t>Indigo</t>
+  </si>
+  <si>
+    <t>#4F46E5</t>
+  </si>
+  <si>
+    <t>Secondary</t>
+  </si>
+  <si>
+    <t>Cyan</t>
+  </si>
+  <si>
+    <t>#06B6D4</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>#22C55E</t>
+  </si>
+  <si>
+    <t>Warning</t>
+  </si>
+  <si>
+    <t>Amber</t>
+  </si>
+  <si>
+    <t>#F59E0B</t>
+  </si>
+  <si>
+    <t>Background</t>
+  </si>
+  <si>
+    <t>Light Gray</t>
+  </si>
+  <si>
+    <t>#F8FAFC</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Dark Slate</t>
+  </si>
+  <si>
+    <t>#0F172A</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>Element</t>
+  </si>
+  <si>
+    <t>Cover Title</t>
+  </si>
+  <si>
+    <t>Main Headings (H1)</t>
+  </si>
+  <si>
+    <t>Sub Headings (H2)</t>
+  </si>
+  <si>
+    <t>Normal Text</t>
+  </si>
+  <si>
+    <t>Table Headers</t>
+  </si>
+  <si>
+    <t>Table Header Text</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>#FFFFFF</t>
+  </si>
+  <si>
+    <t>Table Borders</t>
+  </si>
+  <si>
+    <t>Gray</t>
+  </si>
+  <si>
+    <t>#CBD5E1</t>
+  </si>
+  <si>
+    <t>Notes / Future Enhancements</t>
+  </si>
+  <si>
+    <t>Page Background</t>
+  </si>
+  <si>
+    <t>Primary Heading      : #4F46E5</t>
+  </si>
+  <si>
+    <t>Sub Heading          : #06B6D4</t>
+  </si>
+  <si>
+    <t>Body Text            : #0F172A</t>
+  </si>
+  <si>
+    <t>Table Header         : #4F46E5</t>
+  </si>
+  <si>
+    <t>Table Border         : #CBD5E1</t>
+  </si>
+  <si>
+    <t>Future Enhancements  : #F59E0B</t>
+  </si>
+  <si>
+    <t>Background           : #FFFFFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EduFlow AI Phase 1 TimeLine </t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Creating Functional Requirements for the Project</t>
+  </si>
+  <si>
+    <t>Rough Sketching of the Project Workflow</t>
+  </si>
+  <si>
+    <t>Database Structure Design</t>
+  </si>
+  <si>
+    <t>UI / UX Design using Google Stitch and Figma</t>
+  </si>
+  <si>
+    <t>Designing Phase</t>
+  </si>
+  <si>
+    <t>Finalize the Project Design</t>
+  </si>
+  <si>
+    <t>Frontend Project Setup (React + Routing)</t>
+  </si>
+  <si>
+    <t>Frontend Development</t>
+  </si>
+  <si>
+    <t>Authentication Screens (Login, Register, Forgot Password)</t>
+  </si>
+  <si>
+    <t>Dashboard, Goals, Tasks and Analytics UI</t>
+  </si>
+  <si>
+    <t>Profile Management and Calendar View UI</t>
+  </si>
+  <si>
+    <t>Backend Project Setup (.NET Core 8 + Architecture)</t>
+  </si>
+  <si>
+    <t>Backend Development</t>
+  </si>
+  <si>
+    <t>Authentication APIs (Login, Register, Forgot Password)</t>
+  </si>
+  <si>
+    <t>Goal Management, Task Management and User Profile APIs</t>
+  </si>
+  <si>
+    <t>Planner Engine V1 and Schedule Generation</t>
+  </si>
+  <si>
+    <t>Core Development</t>
+  </si>
+  <si>
+    <t>Dashboard Integration and Calendar Integration</t>
+  </si>
+  <si>
+    <t>Integration Phase</t>
+  </si>
+  <si>
+    <t>Testing and Bug Fixing</t>
+  </si>
+  <si>
+    <t>Testing Phase</t>
+  </si>
+  <si>
+    <t>Total Tasks</t>
+  </si>
+  <si>
+    <t>Completion %</t>
   </si>
 </sst>
 </file>
@@ -258,7 +448,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -289,8 +479,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -322,11 +542,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -342,18 +577,47 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -363,10 +627,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFEF3C7"/>
+      <color rgb="FFF59E0B"/>
       <color rgb="FF06B6D4"/>
       <color rgb="FF4F46E5"/>
-      <color rgb="FFF59E0B"/>
-      <color rgb="FFFEF3C7"/>
     </mruColors>
   </colors>
   <extLst>
@@ -755,7 +1019,7 @@
         <v>15</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -774,169 +1038,169 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
+      <c r="A1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>35</v>
-      </c>
       <c r="C8" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -966,65 +1230,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="9"/>
+      <c r="A1" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="8"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1036,172 +1300,640 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ED9154C-93DA-44CF-8778-E92970739FE3}">
+  <dimension ref="A2:N11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L6" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="J9" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="L9" s="12" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="J10" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="J11" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5CB8FFB-371A-48FE-B0A8-736AABF270A1}">
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.6640625" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A1" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+    </row>
+    <row r="6" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="E6" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+    </row>
+    <row r="7" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>1</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="D7" s="14">
+        <v>46189</v>
+      </c>
+      <c r="E7" s="14">
+        <v>46190</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="H7" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="I7" s="16">
+        <f>COUNTA(B7:B21)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>2</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="14">
+        <v>46191</v>
+      </c>
+      <c r="E8" s="14">
+        <v>46191</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="H8" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="I8" s="17">
+        <f>COUNTIF(F7:F21,"Completed")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
-        <v>1</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="7">
-        <v>46189</v>
-      </c>
-      <c r="E5" s="7">
-        <v>46190</v>
-      </c>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>2</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="7">
-        <v>46191</v>
-      </c>
-      <c r="E6" s="7">
-        <v>46191</v>
-      </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="7">
+      <c r="D9" s="14">
         <v>46192</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E9" s="14">
         <v>46193</v>
       </c>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
-        <v>3</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" s="7">
+      <c r="F9" s="5"/>
+      <c r="H9" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" s="18">
+        <f>COUNTIF(F7:F21,"In Progress")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>4</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="14">
         <v>46193</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E10" s="14">
         <v>46200</v>
       </c>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
-        <v>4</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" s="7">
+      <c r="F10" s="5"/>
+      <c r="H10" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" s="19">
+        <f>COUNTIF(F7:F21,Planned)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>5</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="14">
         <v>46201</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E11" s="14">
         <v>46202</v>
       </c>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="F11" s="5"/>
+      <c r="H11" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="I11" s="20">
+        <f>COUNTIF(F8:F22,"Completed")/COUNTA(B8:B22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>6</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" s="14">
+        <v>46203</v>
+      </c>
+      <c r="E12" s="14">
+        <v>46203</v>
+      </c>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" s="5">
+        <v>7</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="14">
+        <v>46204</v>
+      </c>
+      <c r="E13" s="14">
+        <v>46204</v>
+      </c>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" s="5">
+        <v>8</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D14" s="14">
+        <v>46205</v>
+      </c>
+      <c r="E14" s="14">
+        <v>46206</v>
+      </c>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" s="5">
+        <v>9</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D15" s="14">
+        <v>46207</v>
+      </c>
+      <c r="E15" s="14">
+        <v>46207</v>
+      </c>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" s="5">
+        <v>10</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" s="14">
+        <v>46208</v>
+      </c>
+      <c r="E16" s="14">
+        <v>46208</v>
+      </c>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
+        <v>11</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" s="14">
+        <v>46209</v>
+      </c>
+      <c r="E17" s="14">
+        <v>46209</v>
+      </c>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="5">
+        <v>12</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" s="14">
+        <v>46210</v>
+      </c>
+      <c r="E18" s="14">
+        <v>46211</v>
+      </c>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="5">
+        <v>13</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D19" s="14">
+        <v>46212</v>
+      </c>
+      <c r="E19" s="14">
+        <v>46221</v>
+      </c>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="5">
+        <v>14</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" s="14">
+        <v>46222</v>
+      </c>
+      <c r="E20" s="14">
+        <v>46223</v>
+      </c>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="5">
+        <v>15</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="14">
+        <v>46224</v>
+      </c>
+      <c r="E21" s="14">
+        <v>46225</v>
+      </c>
+      <c r="F21" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A5:F5"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:F21" xr:uid="{2BA7D6B5-8642-45FA-AE77-6AD981377E68}">
+      <formula1>"Not Started,Started,Planned,In Progress,Research,Completed,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
commit changes and added workflow of the project
</commit_message>
<xml_diff>
--- a/docs/EduFlow AI Details.xlsx
+++ b/docs/EduFlow AI Details.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0885FAB1-9EA8-47B3-AEAE-EEB05076DA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="4" xr2:uid="{92BD4C14-6350-41A2-989D-BE19952A9F2F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{92BD4C14-6350-41A2-989D-BE19952A9F2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -617,16 +617,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1127,16 +1127,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
@@ -1319,10 +1319,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="19"/>
+      <c r="B1" s="21"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
@@ -1658,37 +1658,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="18"/>
+      <c r="Q1" s="18"/>
+      <c r="R1" s="18"/>
     </row>
     <row r="5" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
     </row>
     <row r="6" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">

</xml_diff>